<commit_message>
feat: Parte 2 do guia com passo a passo detalhado (11 fichas)
Endereços oficiais dos escritórios da DNM e da Oficina de Expedição,
escribanía, antecedentes para estrangeiros, Interpol e requisitos da
cédula (Res. 717/2026). Atualiza mapa, cronograma, checklists, planilha
e o arquivo único para o Codex.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016nuk5WywdRsNVK1A3CDfL6
</commit_message>
<xml_diff>
--- a/entregavel-paraguai-30-dias/planilha-custos-mudanca-paraguai.xlsx
+++ b/entregavel-paraguai-30-dias/planilha-custos-mudanca-paraguai.xlsx
@@ -2126,7 +2126,7 @@
       </c>
       <c r="B19" s="22" t="inlineStr">
         <is>
-          <t>Cópias autenticadas / escribanía (se pedirem)</t>
+          <t>Cópias autenticadas na escribanía (4 por pessoa)</t>
         </is>
       </c>
       <c r="C19" s="23" t="inlineStr">
@@ -2135,8 +2135,9 @@
         </is>
       </c>
       <c r="D19" s="24" t="n"/>
-      <c r="E19" s="23" t="n">
-        <v>0</v>
+      <c r="E19" s="21">
+        <f>Pessoas*4</f>
+        <v/>
       </c>
       <c r="F19" s="25">
         <f>IF(D19="","",IF(C19="R$",D19*E19,IF(C19="Gs",D19*E19/GsPorReal,IF(C19="US$",D19*E19*GsPorDolar/GsPorReal,""))))</f>
@@ -2154,7 +2155,7 @@
       </c>
       <c r="J19" s="22" t="inlineStr">
         <is>
-          <t>Escribanía local</t>
+          <t>Escribanía local — pergunte o valor por cópia</t>
         </is>
       </c>
     </row>

</xml_diff>